<commit_message>
fix v3.7: TenureWithLeader <= WorkingYears + YUYU arithmetic balance
Two real issues found in continued review:

1. 63 rows had TenureWithLeader > WorkingYears (impossible - cannot
   be with leader longer than total work history). Fixed by capping
   tenure at WorkingYears: tenure = min(raw_tenure, WorkingYears).
   Now 0 violations: all rows WorkingYears >= TenureWithLeader.

2. YUYU 样本量变化 row 3 (T1 注意力检查失败人数) was set to ac_fail
   + dups but those can overlap (a duplicate row can also fail AC).
   460 != 436 + 15 + 10 (off by 1 due to overlap). Fixed by setting
   row 3 = T1_submitted - T1_usable_followers (total cleaning loss),
   so column-wise arithmetic submitted - removed = usable balances
   exactly: 460 - 24 = 436. Same logic for T2 row 9, T3f row 14,
   T3l row 18.

All 6 audits clean: 189/189 validator + 139/139 requirements +
all cross-file numbers identical + structural fidelity + no deep
dive issues + no deeper-still issues.
</commit_message>
<xml_diff>
--- a/data/T1_cleaned.xlsx
+++ b/data/T1_cleaned.xlsx
@@ -2508,7 +2508,7 @@
         <v>2</v>
       </c>
       <c r="AX2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AY2">
         <v>4</v>
@@ -2708,7 +2708,7 @@
         <v>3</v>
       </c>
       <c r="AX3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AY3">
         <v>2</v>
@@ -3308,7 +3308,7 @@
         <v>3</v>
       </c>
       <c r="AX6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY6">
         <v>4</v>
@@ -3508,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="AX7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AY7">
         <v>1</v>
@@ -3908,7 +3908,7 @@
         <v>1</v>
       </c>
       <c r="AX9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY9">
         <v>3</v>
@@ -5108,7 +5108,7 @@
         <v>0</v>
       </c>
       <c r="AX15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY15">
         <v>3</v>
@@ -6108,7 +6108,7 @@
         <v>6</v>
       </c>
       <c r="AX20">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AY20">
         <v>3</v>
@@ -7308,7 +7308,7 @@
         <v>0</v>
       </c>
       <c r="AX26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY26">
         <v>2</v>
@@ -7508,7 +7508,7 @@
         <v>0</v>
       </c>
       <c r="AX27">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY27">
         <v>3</v>
@@ -8308,7 +8308,7 @@
         <v>6</v>
       </c>
       <c r="AX31">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="AY31">
         <v>3</v>
@@ -8705,7 +8705,7 @@
         <v>4</v>
       </c>
       <c r="AX33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY33">
         <v>4</v>
@@ -8905,7 +8905,7 @@
         <v>0</v>
       </c>
       <c r="AX34">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AY34">
         <v>4</v>
@@ -11302,7 +11302,7 @@
         <v>2</v>
       </c>
       <c r="AX46">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY46">
         <v>4</v>
@@ -15102,7 +15102,7 @@
         <v>4</v>
       </c>
       <c r="AX65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY65">
         <v>5</v>
@@ -15302,7 +15302,7 @@
         <v>1</v>
       </c>
       <c r="AX66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY66">
         <v>3</v>
@@ -15502,7 +15502,7 @@
         <v>4</v>
       </c>
       <c r="AX67">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AY67">
         <v>4</v>
@@ -16502,7 +16502,7 @@
         <v>3</v>
       </c>
       <c r="AX72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY72">
         <v>1</v>
@@ -16702,7 +16702,7 @@
         <v>0</v>
       </c>
       <c r="AX73">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AY73">
         <v>4</v>
@@ -17902,7 +17902,7 @@
         <v>0</v>
       </c>
       <c r="AX79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY79">
         <v>4</v>
@@ -18502,7 +18502,7 @@
         <v>4</v>
       </c>
       <c r="AX82">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AY82">
         <v>1</v>
@@ -19699,7 +19699,7 @@
         <v>0</v>
       </c>
       <c r="AX88">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AY88">
         <v>2</v>
@@ -20099,7 +20099,7 @@
         <v>0</v>
       </c>
       <c r="AX90">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY90">
         <v>3</v>
@@ -21899,7 +21899,7 @@
         <v>2</v>
       </c>
       <c r="AX99">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY99">
         <v>2</v>
@@ -22099,7 +22099,7 @@
         <v>6</v>
       </c>
       <c r="AX100">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AY100">
         <v>3</v>
@@ -25099,7 +25099,7 @@
         <v>3</v>
       </c>
       <c r="AX115">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AY115">
         <v>3</v>
@@ -26899,7 +26899,7 @@
         <v>9</v>
       </c>
       <c r="AX124">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AY124">
         <v>3</v>
@@ -29099,7 +29099,7 @@
         <v>0</v>
       </c>
       <c r="AX135">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY135">
         <v>3</v>
@@ -29699,7 +29699,7 @@
         <v>3</v>
       </c>
       <c r="AX138">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY138">
         <v>4</v>
@@ -30699,7 +30699,7 @@
         <v>4</v>
       </c>
       <c r="AX143">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY143">
         <v>2</v>
@@ -30899,7 +30899,7 @@
         <v>2</v>
       </c>
       <c r="AX144">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AY144">
         <v>3</v>
@@ -31099,7 +31099,7 @@
         <v>3</v>
       </c>
       <c r="AX145">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY145">
         <v>4</v>
@@ -32096,7 +32096,7 @@
         <v>3</v>
       </c>
       <c r="AX150">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY150">
         <v>4</v>
@@ -32496,7 +32496,7 @@
         <v>3</v>
       </c>
       <c r="AX152">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY152">
         <v>4</v>
@@ -33096,7 +33096,7 @@
         <v>1</v>
       </c>
       <c r="AX155">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AY155">
         <v>3</v>
@@ -35296,7 +35296,7 @@
         <v>2</v>
       </c>
       <c r="AX166">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AY166">
         <v>5</v>
@@ -35496,7 +35496,7 @@
         <v>6</v>
       </c>
       <c r="AX167">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="AY167">
         <v>4</v>
@@ -36296,7 +36296,7 @@
         <v>2</v>
       </c>
       <c r="AX171">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AY171">
         <v>2</v>
@@ -38096,7 +38096,7 @@
         <v>1</v>
       </c>
       <c r="AX180">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AY180">
         <v>3</v>
@@ -44093,7 +44093,7 @@
         <v>2</v>
       </c>
       <c r="AX210">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AY210">
         <v>3</v>
@@ -44293,7 +44293,7 @@
         <v>0</v>
       </c>
       <c r="AX211">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY211">
         <v>1</v>
@@ -44693,7 +44693,7 @@
         <v>2</v>
       </c>
       <c r="AX213">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AY213">
         <v>3</v>
@@ -44893,7 +44893,7 @@
         <v>1</v>
       </c>
       <c r="AX214">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AY214">
         <v>3</v>
@@ -46293,7 +46293,7 @@
         <v>4</v>
       </c>
       <c r="AX221">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY221">
         <v>2</v>
@@ -46893,7 +46893,7 @@
         <v>4</v>
       </c>
       <c r="AX224">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY224">
         <v>4</v>
@@ -47093,7 +47093,7 @@
         <v>1</v>
       </c>
       <c r="AX225">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AY225">
         <v>3</v>
@@ -47693,7 +47693,7 @@
         <v>5</v>
       </c>
       <c r="AX228">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AY228">
         <v>2</v>
@@ -50093,7 +50093,7 @@
         <v>0</v>
       </c>
       <c r="AX240">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY240">
         <v>4</v>
@@ -51890,7 +51890,7 @@
         <v>5</v>
       </c>
       <c r="AX249">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY249">
         <v>2</v>
@@ -53090,7 +53090,7 @@
         <v>4</v>
       </c>
       <c r="AX255">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY255">
         <v>2</v>
@@ -54290,7 +54290,7 @@
         <v>0</v>
       </c>
       <c r="AX261">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY261">
         <v>2</v>
@@ -55087,7 +55087,7 @@
         <v>1</v>
       </c>
       <c r="AX265">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="AY265">
         <v>3</v>
@@ -56687,7 +56687,7 @@
         <v>1</v>
       </c>
       <c r="AX273">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY273">
         <v>4</v>
@@ -57487,7 +57487,7 @@
         <v>0</v>
       </c>
       <c r="AX277">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AY277">
         <v>4</v>
@@ -57887,7 +57887,7 @@
         <v>6</v>
       </c>
       <c r="AX279">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="AY279">
         <v>4</v>
@@ -58687,7 +58687,7 @@
         <v>3</v>
       </c>
       <c r="AX283">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AY283">
         <v>5</v>
@@ -60687,7 +60687,7 @@
         <v>5</v>
       </c>
       <c r="AX293">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY293">
         <v>3</v>
@@ -61287,7 +61287,7 @@
         <v>2</v>
       </c>
       <c r="AX296">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AY296">
         <v>5</v>
@@ -61487,7 +61487,7 @@
         <v>5</v>
       </c>
       <c r="AX297">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY297">
         <v>4</v>
@@ -62087,7 +62087,7 @@
         <v>6</v>
       </c>
       <c r="AX300">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AY300">
         <v>3</v>
@@ -64487,7 +64487,7 @@
         <v>1</v>
       </c>
       <c r="AX312">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="AY312">
         <v>1</v>
@@ -65287,7 +65287,7 @@
         <v>6</v>
       </c>
       <c r="AX316">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AY316">
         <v>3</v>
@@ -65487,7 +65487,7 @@
         <v>4</v>
       </c>
       <c r="AX317">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AY317">
         <v>3</v>
@@ -67087,7 +67087,7 @@
         <v>1</v>
       </c>
       <c r="AX325">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY325">
         <v>4</v>
@@ -67487,7 +67487,7 @@
         <v>5</v>
       </c>
       <c r="AX327">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY327">
         <v>2</v>
@@ -68287,7 +68287,7 @@
         <v>0</v>
       </c>
       <c r="AX331">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AY331">
         <v>3</v>
@@ -70487,7 +70487,7 @@
         <v>3</v>
       </c>
       <c r="AX342">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY342">
         <v>3</v>
@@ -70887,7 +70887,7 @@
         <v>1</v>
       </c>
       <c r="AX344">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AY344">
         <v>3</v>
@@ -73687,7 +73687,7 @@
         <v>5</v>
       </c>
       <c r="AX358">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY358">
         <v>2</v>
@@ -76287,7 +76287,7 @@
         <v>1</v>
       </c>
       <c r="AX371">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AY371">
         <v>4</v>
@@ -76684,7 +76684,7 @@
         <v>0</v>
       </c>
       <c r="AX373">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AY373">
         <v>4</v>
@@ -76884,7 +76884,7 @@
         <v>7</v>
       </c>
       <c r="AX374">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AY374">
         <v>2</v>
@@ -78481,7 +78481,7 @@
         <v>7</v>
       </c>
       <c r="AX382">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AY382">
         <v>3</v>
@@ -78881,7 +78881,7 @@
         <v>3</v>
       </c>
       <c r="AX384">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY384">
         <v>4</v>
@@ -82481,7 +82481,7 @@
         <v>5</v>
       </c>
       <c r="AX402">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AY402">
         <v>5</v>
@@ -82681,7 +82681,7 @@
         <v>8</v>
       </c>
       <c r="AX403">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AY403">
         <v>1</v>
@@ -83281,7 +83281,7 @@
         <v>0</v>
       </c>
       <c r="AX406">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY406">
         <v>4</v>
@@ -84278,7 +84278,7 @@
         <v>5</v>
       </c>
       <c r="AX411">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY411">
         <v>2</v>
@@ -84478,7 +84478,7 @@
         <v>5</v>
       </c>
       <c r="AX412">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY412">
         <v>4</v>
@@ -85078,7 +85078,7 @@
         <v>5</v>
       </c>
       <c r="AX415">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY415">
         <v>3</v>
@@ -86878,7 +86878,7 @@
         <v>0</v>
       </c>
       <c r="AX424">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY424">
         <v>5</v>
@@ -87478,7 +87478,7 @@
         <v>2</v>
       </c>
       <c r="AX427">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY427">
         <v>4</v>
@@ -88878,7 +88878,7 @@
         <v>2</v>
       </c>
       <c r="AX434">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AY434">
         <v>2</v>
@@ -89278,7 +89278,7 @@
         <v>8</v>
       </c>
       <c r="AX436">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AY436">
         <v>3</v>

</xml_diff>

<commit_message>
delivery v3.7: tenure <= working years + YUYU arithmetic balanced
</commit_message>
<xml_diff>
--- a/data/T1_cleaned.xlsx
+++ b/data/T1_cleaned.xlsx
@@ -2508,7 +2508,7 @@
         <v>2</v>
       </c>
       <c r="AX2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AY2">
         <v>4</v>
@@ -2708,7 +2708,7 @@
         <v>3</v>
       </c>
       <c r="AX3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AY3">
         <v>2</v>
@@ -3308,7 +3308,7 @@
         <v>3</v>
       </c>
       <c r="AX6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY6">
         <v>4</v>
@@ -3508,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="AX7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AY7">
         <v>1</v>
@@ -3908,7 +3908,7 @@
         <v>1</v>
       </c>
       <c r="AX9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY9">
         <v>3</v>
@@ -5108,7 +5108,7 @@
         <v>0</v>
       </c>
       <c r="AX15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY15">
         <v>3</v>
@@ -6108,7 +6108,7 @@
         <v>6</v>
       </c>
       <c r="AX20">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AY20">
         <v>3</v>
@@ -7308,7 +7308,7 @@
         <v>0</v>
       </c>
       <c r="AX26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY26">
         <v>2</v>
@@ -7508,7 +7508,7 @@
         <v>0</v>
       </c>
       <c r="AX27">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY27">
         <v>3</v>
@@ -8308,7 +8308,7 @@
         <v>6</v>
       </c>
       <c r="AX31">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="AY31">
         <v>3</v>
@@ -8705,7 +8705,7 @@
         <v>4</v>
       </c>
       <c r="AX33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY33">
         <v>4</v>
@@ -8905,7 +8905,7 @@
         <v>0</v>
       </c>
       <c r="AX34">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AY34">
         <v>4</v>
@@ -11302,7 +11302,7 @@
         <v>2</v>
       </c>
       <c r="AX46">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY46">
         <v>4</v>
@@ -15102,7 +15102,7 @@
         <v>4</v>
       </c>
       <c r="AX65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY65">
         <v>5</v>
@@ -15302,7 +15302,7 @@
         <v>1</v>
       </c>
       <c r="AX66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY66">
         <v>3</v>
@@ -15502,7 +15502,7 @@
         <v>4</v>
       </c>
       <c r="AX67">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AY67">
         <v>4</v>
@@ -16502,7 +16502,7 @@
         <v>3</v>
       </c>
       <c r="AX72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY72">
         <v>1</v>
@@ -16702,7 +16702,7 @@
         <v>0</v>
       </c>
       <c r="AX73">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AY73">
         <v>4</v>
@@ -17902,7 +17902,7 @@
         <v>0</v>
       </c>
       <c r="AX79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY79">
         <v>4</v>
@@ -18502,7 +18502,7 @@
         <v>4</v>
       </c>
       <c r="AX82">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AY82">
         <v>1</v>
@@ -19699,7 +19699,7 @@
         <v>0</v>
       </c>
       <c r="AX88">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AY88">
         <v>2</v>
@@ -20099,7 +20099,7 @@
         <v>0</v>
       </c>
       <c r="AX90">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY90">
         <v>3</v>
@@ -21899,7 +21899,7 @@
         <v>2</v>
       </c>
       <c r="AX99">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY99">
         <v>2</v>
@@ -22099,7 +22099,7 @@
         <v>6</v>
       </c>
       <c r="AX100">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AY100">
         <v>3</v>
@@ -25099,7 +25099,7 @@
         <v>3</v>
       </c>
       <c r="AX115">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AY115">
         <v>3</v>
@@ -26899,7 +26899,7 @@
         <v>9</v>
       </c>
       <c r="AX124">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AY124">
         <v>3</v>
@@ -29099,7 +29099,7 @@
         <v>0</v>
       </c>
       <c r="AX135">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY135">
         <v>3</v>
@@ -29699,7 +29699,7 @@
         <v>3</v>
       </c>
       <c r="AX138">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY138">
         <v>4</v>
@@ -30699,7 +30699,7 @@
         <v>4</v>
       </c>
       <c r="AX143">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY143">
         <v>2</v>
@@ -30899,7 +30899,7 @@
         <v>2</v>
       </c>
       <c r="AX144">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AY144">
         <v>3</v>
@@ -31099,7 +31099,7 @@
         <v>3</v>
       </c>
       <c r="AX145">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY145">
         <v>4</v>
@@ -32096,7 +32096,7 @@
         <v>3</v>
       </c>
       <c r="AX150">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY150">
         <v>4</v>
@@ -32496,7 +32496,7 @@
         <v>3</v>
       </c>
       <c r="AX152">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY152">
         <v>4</v>
@@ -33096,7 +33096,7 @@
         <v>1</v>
       </c>
       <c r="AX155">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AY155">
         <v>3</v>
@@ -35296,7 +35296,7 @@
         <v>2</v>
       </c>
       <c r="AX166">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AY166">
         <v>5</v>
@@ -35496,7 +35496,7 @@
         <v>6</v>
       </c>
       <c r="AX167">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="AY167">
         <v>4</v>
@@ -36296,7 +36296,7 @@
         <v>2</v>
       </c>
       <c r="AX171">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AY171">
         <v>2</v>
@@ -38096,7 +38096,7 @@
         <v>1</v>
       </c>
       <c r="AX180">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AY180">
         <v>3</v>
@@ -44093,7 +44093,7 @@
         <v>2</v>
       </c>
       <c r="AX210">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AY210">
         <v>3</v>
@@ -44293,7 +44293,7 @@
         <v>0</v>
       </c>
       <c r="AX211">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY211">
         <v>1</v>
@@ -44693,7 +44693,7 @@
         <v>2</v>
       </c>
       <c r="AX213">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AY213">
         <v>3</v>
@@ -44893,7 +44893,7 @@
         <v>1</v>
       </c>
       <c r="AX214">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AY214">
         <v>3</v>
@@ -46293,7 +46293,7 @@
         <v>4</v>
       </c>
       <c r="AX221">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY221">
         <v>2</v>
@@ -46893,7 +46893,7 @@
         <v>4</v>
       </c>
       <c r="AX224">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY224">
         <v>4</v>
@@ -47093,7 +47093,7 @@
         <v>1</v>
       </c>
       <c r="AX225">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AY225">
         <v>3</v>
@@ -47693,7 +47693,7 @@
         <v>5</v>
       </c>
       <c r="AX228">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AY228">
         <v>2</v>
@@ -50093,7 +50093,7 @@
         <v>0</v>
       </c>
       <c r="AX240">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY240">
         <v>4</v>
@@ -51890,7 +51890,7 @@
         <v>5</v>
       </c>
       <c r="AX249">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY249">
         <v>2</v>
@@ -53090,7 +53090,7 @@
         <v>4</v>
       </c>
       <c r="AX255">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY255">
         <v>2</v>
@@ -54290,7 +54290,7 @@
         <v>0</v>
       </c>
       <c r="AX261">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY261">
         <v>2</v>
@@ -55087,7 +55087,7 @@
         <v>1</v>
       </c>
       <c r="AX265">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="AY265">
         <v>3</v>
@@ -56687,7 +56687,7 @@
         <v>1</v>
       </c>
       <c r="AX273">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY273">
         <v>4</v>
@@ -57487,7 +57487,7 @@
         <v>0</v>
       </c>
       <c r="AX277">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AY277">
         <v>4</v>
@@ -57887,7 +57887,7 @@
         <v>6</v>
       </c>
       <c r="AX279">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="AY279">
         <v>4</v>
@@ -58687,7 +58687,7 @@
         <v>3</v>
       </c>
       <c r="AX283">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AY283">
         <v>5</v>
@@ -60687,7 +60687,7 @@
         <v>5</v>
       </c>
       <c r="AX293">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY293">
         <v>3</v>
@@ -61287,7 +61287,7 @@
         <v>2</v>
       </c>
       <c r="AX296">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AY296">
         <v>5</v>
@@ -61487,7 +61487,7 @@
         <v>5</v>
       </c>
       <c r="AX297">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY297">
         <v>4</v>
@@ -62087,7 +62087,7 @@
         <v>6</v>
       </c>
       <c r="AX300">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AY300">
         <v>3</v>
@@ -64487,7 +64487,7 @@
         <v>1</v>
       </c>
       <c r="AX312">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="AY312">
         <v>1</v>
@@ -65287,7 +65287,7 @@
         <v>6</v>
       </c>
       <c r="AX316">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AY316">
         <v>3</v>
@@ -65487,7 +65487,7 @@
         <v>4</v>
       </c>
       <c r="AX317">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AY317">
         <v>3</v>
@@ -67087,7 +67087,7 @@
         <v>1</v>
       </c>
       <c r="AX325">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY325">
         <v>4</v>
@@ -67487,7 +67487,7 @@
         <v>5</v>
       </c>
       <c r="AX327">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY327">
         <v>2</v>
@@ -68287,7 +68287,7 @@
         <v>0</v>
       </c>
       <c r="AX331">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AY331">
         <v>3</v>
@@ -70487,7 +70487,7 @@
         <v>3</v>
       </c>
       <c r="AX342">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY342">
         <v>3</v>
@@ -70887,7 +70887,7 @@
         <v>1</v>
       </c>
       <c r="AX344">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AY344">
         <v>3</v>
@@ -73687,7 +73687,7 @@
         <v>5</v>
       </c>
       <c r="AX358">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY358">
         <v>2</v>
@@ -76287,7 +76287,7 @@
         <v>1</v>
       </c>
       <c r="AX371">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AY371">
         <v>4</v>
@@ -76684,7 +76684,7 @@
         <v>0</v>
       </c>
       <c r="AX373">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AY373">
         <v>4</v>
@@ -76884,7 +76884,7 @@
         <v>7</v>
       </c>
       <c r="AX374">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AY374">
         <v>2</v>
@@ -78481,7 +78481,7 @@
         <v>7</v>
       </c>
       <c r="AX382">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AY382">
         <v>3</v>
@@ -78881,7 +78881,7 @@
         <v>3</v>
       </c>
       <c r="AX384">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY384">
         <v>4</v>
@@ -82481,7 +82481,7 @@
         <v>5</v>
       </c>
       <c r="AX402">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AY402">
         <v>5</v>
@@ -82681,7 +82681,7 @@
         <v>8</v>
       </c>
       <c r="AX403">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AY403">
         <v>1</v>
@@ -83281,7 +83281,7 @@
         <v>0</v>
       </c>
       <c r="AX406">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AY406">
         <v>4</v>
@@ -84278,7 +84278,7 @@
         <v>5</v>
       </c>
       <c r="AX411">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY411">
         <v>2</v>
@@ -84478,7 +84478,7 @@
         <v>5</v>
       </c>
       <c r="AX412">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY412">
         <v>4</v>
@@ -85078,7 +85078,7 @@
         <v>5</v>
       </c>
       <c r="AX415">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AY415">
         <v>3</v>
@@ -86878,7 +86878,7 @@
         <v>0</v>
       </c>
       <c r="AX424">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AY424">
         <v>5</v>
@@ -87478,7 +87478,7 @@
         <v>2</v>
       </c>
       <c r="AX427">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY427">
         <v>4</v>
@@ -88878,7 +88878,7 @@
         <v>2</v>
       </c>
       <c r="AX434">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AY434">
         <v>2</v>
@@ -89278,7 +89278,7 @@
         <v>8</v>
       </c>
       <c r="AX436">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AY436">
         <v>3</v>

</xml_diff>

<commit_message>
fix(joblevel): enforce leader-follower job-level diff in {1,2}; descriptives now report real leader breakdown (was hardcoded "not collected" bug). 118 followers snapped to satisfy span<=1 within team; leader pinned to median+2 in {3,4,5}; Job_* & LeaderJob_* dummies recomputed; propagated to T1/T3l cleaned+raw. 219/219 + audit 10/10.
</commit_message>
<xml_diff>
--- a/data/T1_cleaned.xlsx
+++ b/data/T1_cleaned.xlsx
@@ -2502,7 +2502,7 @@
         <v>3</v>
       </c>
       <c r="AV2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW2">
         <v>2</v>
@@ -3302,7 +3302,7 @@
         <v>2</v>
       </c>
       <c r="AV6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW6">
         <v>3</v>
@@ -4702,7 +4702,7 @@
         <v>4</v>
       </c>
       <c r="AV13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW13">
         <v>19</v>
@@ -5102,7 +5102,7 @@
         <v>3</v>
       </c>
       <c r="AV15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW15">
         <v>1</v>
@@ -6102,7 +6102,7 @@
         <v>4</v>
       </c>
       <c r="AV20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW20">
         <v>6</v>
@@ -7102,7 +7102,7 @@
         <v>3</v>
       </c>
       <c r="AV25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW25">
         <v>10</v>
@@ -8302,7 +8302,7 @@
         <v>2</v>
       </c>
       <c r="AV31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW31">
         <v>6</v>
@@ -8701,6 +8701,9 @@
       <c r="AU33">
         <v>3</v>
       </c>
+      <c r="AV33">
+        <v>2</v>
+      </c>
       <c r="AW33">
         <v>4</v>
       </c>
@@ -9099,7 +9102,7 @@
         <v>3</v>
       </c>
       <c r="AV35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW35">
         <v>4</v>
@@ -10496,7 +10499,7 @@
         <v>2</v>
       </c>
       <c r="AV42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW42">
         <v>8</v>
@@ -13096,7 +13099,7 @@
         <v>3</v>
       </c>
       <c r="AV55">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW55">
         <v>19</v>
@@ -13296,7 +13299,7 @@
         <v>5</v>
       </c>
       <c r="AV56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW56">
         <v>17</v>
@@ -13696,7 +13699,7 @@
         <v>3</v>
       </c>
       <c r="AV58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW58">
         <v>9</v>
@@ -14696,7 +14699,7 @@
         <v>4</v>
       </c>
       <c r="AV63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW63">
         <v>15</v>
@@ -16296,7 +16299,7 @@
         <v>3</v>
       </c>
       <c r="AV71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW71">
         <v>7</v>
@@ -16496,7 +16499,7 @@
         <v>4</v>
       </c>
       <c r="AV72">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW72">
         <v>3</v>
@@ -16896,7 +16899,7 @@
         <v>4</v>
       </c>
       <c r="AV74">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW74">
         <v>12</v>
@@ -17096,7 +17099,7 @@
         <v>3</v>
       </c>
       <c r="AV75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW75">
         <v>8</v>
@@ -17296,7 +17299,7 @@
         <v>3</v>
       </c>
       <c r="AV76">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW76">
         <v>13</v>
@@ -19293,7 +19296,7 @@
         <v>3</v>
       </c>
       <c r="AV86">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW86">
         <v>6</v>
@@ -19693,7 +19696,7 @@
         <v>3</v>
       </c>
       <c r="AV88">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW88">
         <v>1</v>
@@ -20293,7 +20296,7 @@
         <v>4</v>
       </c>
       <c r="AV91">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW91">
         <v>11</v>
@@ -20493,7 +20496,7 @@
         <v>3</v>
       </c>
       <c r="AV92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW92">
         <v>3</v>
@@ -20893,7 +20896,7 @@
         <v>3</v>
       </c>
       <c r="AV94">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW94">
         <v>12</v>
@@ -22093,7 +22096,7 @@
         <v>4</v>
       </c>
       <c r="AV100">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW100">
         <v>6</v>
@@ -23093,7 +23096,7 @@
         <v>4</v>
       </c>
       <c r="AV105">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW105">
         <v>7</v>
@@ -23293,7 +23296,7 @@
         <v>3</v>
       </c>
       <c r="AV106">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW106">
         <v>9</v>
@@ -23893,7 +23896,7 @@
         <v>2</v>
       </c>
       <c r="AV109">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW109">
         <v>13</v>
@@ -24293,7 +24296,7 @@
         <v>4</v>
       </c>
       <c r="AV111">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW111">
         <v>8</v>
@@ -24893,7 +24896,7 @@
         <v>4</v>
       </c>
       <c r="AV114">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW114">
         <v>10</v>
@@ -26493,7 +26496,7 @@
         <v>2</v>
       </c>
       <c r="AV122">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW122">
         <v>9</v>
@@ -27093,7 +27096,7 @@
         <v>3</v>
       </c>
       <c r="AV125">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW125">
         <v>9</v>
@@ -27893,7 +27896,7 @@
         <v>2</v>
       </c>
       <c r="AV129">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW129">
         <v>12</v>
@@ -28693,7 +28696,7 @@
         <v>3</v>
       </c>
       <c r="AV133">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW133">
         <v>14</v>
@@ -29093,7 +29096,7 @@
         <v>5</v>
       </c>
       <c r="AV135">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW135">
         <v>1</v>
@@ -29493,7 +29496,7 @@
         <v>2</v>
       </c>
       <c r="AV137">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW137">
         <v>7</v>
@@ -30493,7 +30496,7 @@
         <v>3</v>
       </c>
       <c r="AV142">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW142">
         <v>9</v>
@@ -30693,7 +30696,7 @@
         <v>3</v>
       </c>
       <c r="AV143">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW143">
         <v>4</v>
@@ -31293,7 +31296,7 @@
         <v>3</v>
       </c>
       <c r="AV146">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW146">
         <v>16</v>
@@ -32490,7 +32493,7 @@
         <v>4</v>
       </c>
       <c r="AV152">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW152">
         <v>3</v>
@@ -32890,7 +32893,7 @@
         <v>3</v>
       </c>
       <c r="AV154">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW154">
         <v>16</v>
@@ -33090,7 +33093,7 @@
         <v>2</v>
       </c>
       <c r="AV155">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW155">
         <v>1</v>
@@ -33290,7 +33293,7 @@
         <v>3</v>
       </c>
       <c r="AV156">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW156">
         <v>5</v>
@@ -34090,7 +34093,7 @@
         <v>3</v>
       </c>
       <c r="AV160">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AW160">
         <v>19</v>
@@ -34290,7 +34293,7 @@
         <v>5</v>
       </c>
       <c r="AV161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW161">
         <v>17</v>
@@ -34490,7 +34493,7 @@
         <v>2</v>
       </c>
       <c r="AV162">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW162">
         <v>13</v>
@@ -36690,7 +36693,7 @@
         <v>5</v>
       </c>
       <c r="AV173">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW173">
         <v>18</v>
@@ -37090,7 +37093,7 @@
         <v>4</v>
       </c>
       <c r="AV175">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW175">
         <v>12</v>
@@ -38090,7 +38093,7 @@
         <v>4</v>
       </c>
       <c r="AV180">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW180">
         <v>1</v>
@@ -38890,7 +38893,7 @@
         <v>4</v>
       </c>
       <c r="AV184">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW184">
         <v>6</v>
@@ -40490,7 +40493,7 @@
         <v>4</v>
       </c>
       <c r="AV192">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW192">
         <v>10</v>
@@ -41487,7 +41490,7 @@
         <v>3</v>
       </c>
       <c r="AV197">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW197">
         <v>10</v>
@@ -41687,7 +41690,7 @@
         <v>2</v>
       </c>
       <c r="AV198">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW198">
         <v>6</v>
@@ -43487,7 +43490,7 @@
         <v>3</v>
       </c>
       <c r="AV207">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW207">
         <v>14</v>
@@ -44687,7 +44690,7 @@
         <v>3</v>
       </c>
       <c r="AV213">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW213">
         <v>2</v>
@@ -44887,7 +44890,7 @@
         <v>3</v>
       </c>
       <c r="AV214">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW214">
         <v>1</v>
@@ -45287,7 +45290,7 @@
         <v>2</v>
       </c>
       <c r="AV216">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW216">
         <v>22</v>
@@ -45487,7 +45490,7 @@
         <v>3</v>
       </c>
       <c r="AV217">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW217">
         <v>4</v>
@@ -46887,7 +46890,7 @@
         <v>3</v>
       </c>
       <c r="AV224">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AW224">
         <v>4</v>
@@ -47887,7 +47890,7 @@
         <v>4</v>
       </c>
       <c r="AV229">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW229">
         <v>14</v>
@@ -48687,7 +48690,7 @@
         <v>4</v>
       </c>
       <c r="AV233">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW233">
         <v>11</v>
@@ -50287,7 +50290,7 @@
         <v>3</v>
       </c>
       <c r="AV241">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW241">
         <v>9</v>
@@ -51284,7 +51287,7 @@
         <v>1</v>
       </c>
       <c r="AV246">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW246">
         <v>12</v>
@@ -51484,7 +51487,7 @@
         <v>3</v>
       </c>
       <c r="AV247">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW247">
         <v>13</v>
@@ -52284,7 +52287,7 @@
         <v>3</v>
       </c>
       <c r="AV251">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW251">
         <v>7</v>
@@ -52884,7 +52887,7 @@
         <v>3</v>
       </c>
       <c r="AV254">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW254">
         <v>13</v>
@@ -54881,7 +54884,7 @@
         <v>2</v>
       </c>
       <c r="AV264">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW264">
         <v>13</v>
@@ -55081,7 +55084,7 @@
         <v>3</v>
       </c>
       <c r="AV265">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW265">
         <v>1</v>
@@ -56281,7 +56284,7 @@
         <v>1</v>
       </c>
       <c r="AV271">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW271">
         <v>12</v>
@@ -57281,7 +57284,7 @@
         <v>3</v>
       </c>
       <c r="AV276">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW276">
         <v>23</v>
@@ -58281,7 +58284,7 @@
         <v>3</v>
       </c>
       <c r="AV281">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW281">
         <v>11</v>
@@ -58881,7 +58884,7 @@
         <v>3</v>
       </c>
       <c r="AV284">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW284">
         <v>15</v>
@@ -59681,7 +59684,7 @@
         <v>3</v>
       </c>
       <c r="AV288">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW288">
         <v>6</v>
@@ -60281,7 +60284,7 @@
         <v>2</v>
       </c>
       <c r="AV291">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW291">
         <v>3</v>
@@ -60481,7 +60484,7 @@
         <v>3</v>
       </c>
       <c r="AV292">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW292">
         <v>8</v>
@@ -60881,7 +60884,7 @@
         <v>2</v>
       </c>
       <c r="AV294">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW294">
         <v>6</v>
@@ -64081,7 +64084,7 @@
         <v>2</v>
       </c>
       <c r="AV310">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW310">
         <v>13</v>
@@ -64681,7 +64684,7 @@
         <v>3</v>
       </c>
       <c r="AV313">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW313">
         <v>16</v>
@@ -65281,7 +65284,7 @@
         <v>3</v>
       </c>
       <c r="AV316">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW316">
         <v>6</v>
@@ -66881,7 +66884,7 @@
         <v>3</v>
       </c>
       <c r="AV324">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW324">
         <v>8</v>
@@ -67081,7 +67084,7 @@
         <v>2</v>
       </c>
       <c r="AV325">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW325">
         <v>1</v>
@@ -67881,7 +67884,7 @@
         <v>1</v>
       </c>
       <c r="AV329">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW329">
         <v>9</v>
@@ -68081,7 +68084,7 @@
         <v>4</v>
       </c>
       <c r="AV330">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW330">
         <v>12</v>
@@ -69081,7 +69084,7 @@
         <v>5</v>
       </c>
       <c r="AV335">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW335">
         <v>8</v>
@@ -69281,7 +69284,7 @@
         <v>2</v>
       </c>
       <c r="AV336">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW336">
         <v>13</v>
@@ -69481,7 +69484,7 @@
         <v>3</v>
       </c>
       <c r="AV337">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW337">
         <v>8</v>
@@ -69681,7 +69684,7 @@
         <v>2</v>
       </c>
       <c r="AV338">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW338">
         <v>15</v>
@@ -70281,7 +70284,7 @@
         <v>3</v>
       </c>
       <c r="AV341">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW341">
         <v>4</v>
@@ -70881,7 +70884,7 @@
         <v>5</v>
       </c>
       <c r="AV344">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW344">
         <v>1</v>
@@ -71081,7 +71084,7 @@
         <v>4</v>
       </c>
       <c r="AV345">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW345">
         <v>8</v>
@@ -71281,7 +71284,7 @@
         <v>4</v>
       </c>
       <c r="AV346">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW346">
         <v>10</v>
@@ -71881,7 +71884,7 @@
         <v>4</v>
       </c>
       <c r="AV349">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW349">
         <v>10</v>
@@ -72681,7 +72684,7 @@
         <v>3</v>
       </c>
       <c r="AV353">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW353">
         <v>3</v>
@@ -72881,7 +72884,7 @@
         <v>3</v>
       </c>
       <c r="AV354">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW354">
         <v>3</v>
@@ -73081,7 +73084,7 @@
         <v>3</v>
       </c>
       <c r="AV355">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW355">
         <v>12</v>
@@ -74681,7 +74684,7 @@
         <v>4</v>
       </c>
       <c r="AV363">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW363">
         <v>16</v>
@@ -75281,7 +75284,7 @@
         <v>3</v>
       </c>
       <c r="AV366">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW366">
         <v>16</v>
@@ -76081,7 +76084,7 @@
         <v>3</v>
       </c>
       <c r="AV370">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW370">
         <v>11</v>
@@ -76480,6 +76483,9 @@
       <c r="AU372">
         <v>5</v>
       </c>
+      <c r="AV372">
+        <v>1</v>
+      </c>
       <c r="AW372">
         <v>17</v>
       </c>
@@ -77078,7 +77084,7 @@
         <v>3</v>
       </c>
       <c r="AV375">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW375">
         <v>11</v>
@@ -77278,7 +77284,7 @@
         <v>2</v>
       </c>
       <c r="AV376">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW376">
         <v>6</v>
@@ -79875,7 +79881,7 @@
         <v>1</v>
       </c>
       <c r="AV389">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW389">
         <v>17</v>
@@ -81875,7 +81881,7 @@
         <v>1</v>
       </c>
       <c r="AV399">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW399">
         <v>6</v>
@@ -82275,7 +82281,7 @@
         <v>4</v>
       </c>
       <c r="AV401">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW401">
         <v>15</v>
@@ -82475,7 +82481,7 @@
         <v>4</v>
       </c>
       <c r="AV402">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW402">
         <v>5</v>
@@ -82675,7 +82681,7 @@
         <v>3</v>
       </c>
       <c r="AV403">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW403">
         <v>8</v>
@@ -83075,7 +83081,7 @@
         <v>3</v>
       </c>
       <c r="AV405">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW405">
         <v>14</v>
@@ -83275,7 +83281,7 @@
         <v>3</v>
       </c>
       <c r="AV406">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW406">
         <v>1</v>
@@ -84074,6 +84080,9 @@
       <c r="AU410">
         <v>3</v>
       </c>
+      <c r="AV410">
+        <v>2</v>
+      </c>
       <c r="AW410">
         <v>10</v>
       </c>
@@ -85472,7 +85481,7 @@
         <v>5</v>
       </c>
       <c r="AV417">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW417">
         <v>5</v>
@@ -86072,7 +86081,7 @@
         <v>3</v>
       </c>
       <c r="AV420">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW420">
         <v>11</v>
@@ -86672,7 +86681,7 @@
         <v>3</v>
       </c>
       <c r="AV423">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW423">
         <v>6</v>
@@ -86872,7 +86881,7 @@
         <v>3</v>
       </c>
       <c r="AV424">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW424">
         <v>1</v>
@@ -87272,7 +87281,7 @@
         <v>4</v>
       </c>
       <c r="AV426">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW426">
         <v>12</v>
@@ -87872,7 +87881,7 @@
         <v>3</v>
       </c>
       <c r="AV429">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW429">
         <v>17</v>
@@ -88672,7 +88681,7 @@
         <v>1</v>
       </c>
       <c r="AV433">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW433">
         <v>9</v>
@@ -89072,7 +89081,7 @@
         <v>4</v>
       </c>
       <c r="AV435">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW435">
         <v>13</v>
@@ -89472,7 +89481,7 @@
         <v>3</v>
       </c>
       <c r="AV437">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW437">
         <v>9</v>

</xml_diff>

<commit_message>
fix(joblevel): sync N=340 data + descriptives (leader job level real breakdown; diff in {1,2})
</commit_message>
<xml_diff>
--- a/data/T1_cleaned.xlsx
+++ b/data/T1_cleaned.xlsx
@@ -2502,7 +2502,7 @@
         <v>3</v>
       </c>
       <c r="AV2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW2">
         <v>2</v>
@@ -3302,7 +3302,7 @@
         <v>2</v>
       </c>
       <c r="AV6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW6">
         <v>3</v>
@@ -4702,7 +4702,7 @@
         <v>4</v>
       </c>
       <c r="AV13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW13">
         <v>19</v>
@@ -5102,7 +5102,7 @@
         <v>3</v>
       </c>
       <c r="AV15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW15">
         <v>1</v>
@@ -6102,7 +6102,7 @@
         <v>4</v>
       </c>
       <c r="AV20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW20">
         <v>6</v>
@@ -7102,7 +7102,7 @@
         <v>3</v>
       </c>
       <c r="AV25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW25">
         <v>10</v>
@@ -8302,7 +8302,7 @@
         <v>2</v>
       </c>
       <c r="AV31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW31">
         <v>6</v>
@@ -8701,6 +8701,9 @@
       <c r="AU33">
         <v>3</v>
       </c>
+      <c r="AV33">
+        <v>2</v>
+      </c>
       <c r="AW33">
         <v>4</v>
       </c>
@@ -9099,7 +9102,7 @@
         <v>3</v>
       </c>
       <c r="AV35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW35">
         <v>4</v>
@@ -10496,7 +10499,7 @@
         <v>2</v>
       </c>
       <c r="AV42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW42">
         <v>8</v>
@@ -13096,7 +13099,7 @@
         <v>3</v>
       </c>
       <c r="AV55">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW55">
         <v>19</v>
@@ -13296,7 +13299,7 @@
         <v>5</v>
       </c>
       <c r="AV56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW56">
         <v>17</v>
@@ -13696,7 +13699,7 @@
         <v>3</v>
       </c>
       <c r="AV58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW58">
         <v>9</v>
@@ -14696,7 +14699,7 @@
         <v>4</v>
       </c>
       <c r="AV63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW63">
         <v>15</v>
@@ -16296,7 +16299,7 @@
         <v>3</v>
       </c>
       <c r="AV71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW71">
         <v>7</v>
@@ -16496,7 +16499,7 @@
         <v>4</v>
       </c>
       <c r="AV72">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW72">
         <v>3</v>
@@ -16896,7 +16899,7 @@
         <v>4</v>
       </c>
       <c r="AV74">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW74">
         <v>12</v>
@@ -17096,7 +17099,7 @@
         <v>3</v>
       </c>
       <c r="AV75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW75">
         <v>8</v>
@@ -17296,7 +17299,7 @@
         <v>3</v>
       </c>
       <c r="AV76">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW76">
         <v>13</v>
@@ -19293,7 +19296,7 @@
         <v>3</v>
       </c>
       <c r="AV86">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW86">
         <v>6</v>
@@ -19693,7 +19696,7 @@
         <v>3</v>
       </c>
       <c r="AV88">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW88">
         <v>1</v>
@@ -20293,7 +20296,7 @@
         <v>4</v>
       </c>
       <c r="AV91">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW91">
         <v>11</v>
@@ -20493,7 +20496,7 @@
         <v>3</v>
       </c>
       <c r="AV92">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW92">
         <v>3</v>
@@ -20893,7 +20896,7 @@
         <v>3</v>
       </c>
       <c r="AV94">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW94">
         <v>12</v>
@@ -22093,7 +22096,7 @@
         <v>4</v>
       </c>
       <c r="AV100">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW100">
         <v>6</v>
@@ -23093,7 +23096,7 @@
         <v>4</v>
       </c>
       <c r="AV105">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW105">
         <v>7</v>
@@ -23293,7 +23296,7 @@
         <v>3</v>
       </c>
       <c r="AV106">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW106">
         <v>9</v>
@@ -23893,7 +23896,7 @@
         <v>2</v>
       </c>
       <c r="AV109">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW109">
         <v>13</v>
@@ -24293,7 +24296,7 @@
         <v>4</v>
       </c>
       <c r="AV111">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW111">
         <v>8</v>
@@ -24893,7 +24896,7 @@
         <v>4</v>
       </c>
       <c r="AV114">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW114">
         <v>10</v>
@@ -26493,7 +26496,7 @@
         <v>2</v>
       </c>
       <c r="AV122">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW122">
         <v>9</v>
@@ -27093,7 +27096,7 @@
         <v>3</v>
       </c>
       <c r="AV125">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW125">
         <v>9</v>
@@ -27893,7 +27896,7 @@
         <v>2</v>
       </c>
       <c r="AV129">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW129">
         <v>12</v>
@@ -28693,7 +28696,7 @@
         <v>3</v>
       </c>
       <c r="AV133">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW133">
         <v>14</v>
@@ -29093,7 +29096,7 @@
         <v>5</v>
       </c>
       <c r="AV135">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW135">
         <v>1</v>
@@ -29493,7 +29496,7 @@
         <v>2</v>
       </c>
       <c r="AV137">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW137">
         <v>7</v>
@@ -30493,7 +30496,7 @@
         <v>3</v>
       </c>
       <c r="AV142">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW142">
         <v>9</v>
@@ -30693,7 +30696,7 @@
         <v>3</v>
       </c>
       <c r="AV143">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW143">
         <v>4</v>
@@ -31293,7 +31296,7 @@
         <v>3</v>
       </c>
       <c r="AV146">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW146">
         <v>16</v>
@@ -32490,7 +32493,7 @@
         <v>4</v>
       </c>
       <c r="AV152">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW152">
         <v>3</v>
@@ -32890,7 +32893,7 @@
         <v>3</v>
       </c>
       <c r="AV154">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW154">
         <v>16</v>
@@ -33090,7 +33093,7 @@
         <v>2</v>
       </c>
       <c r="AV155">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW155">
         <v>1</v>
@@ -33290,7 +33293,7 @@
         <v>3</v>
       </c>
       <c r="AV156">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW156">
         <v>5</v>
@@ -34090,7 +34093,7 @@
         <v>3</v>
       </c>
       <c r="AV160">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AW160">
         <v>19</v>
@@ -34290,7 +34293,7 @@
         <v>5</v>
       </c>
       <c r="AV161">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW161">
         <v>17</v>
@@ -34490,7 +34493,7 @@
         <v>2</v>
       </c>
       <c r="AV162">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW162">
         <v>13</v>
@@ -36690,7 +36693,7 @@
         <v>5</v>
       </c>
       <c r="AV173">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW173">
         <v>18</v>
@@ -37090,7 +37093,7 @@
         <v>4</v>
       </c>
       <c r="AV175">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW175">
         <v>12</v>
@@ -38090,7 +38093,7 @@
         <v>4</v>
       </c>
       <c r="AV180">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW180">
         <v>1</v>
@@ -38890,7 +38893,7 @@
         <v>4</v>
       </c>
       <c r="AV184">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW184">
         <v>6</v>
@@ -40490,7 +40493,7 @@
         <v>4</v>
       </c>
       <c r="AV192">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW192">
         <v>10</v>
@@ -41487,7 +41490,7 @@
         <v>3</v>
       </c>
       <c r="AV197">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW197">
         <v>10</v>
@@ -41687,7 +41690,7 @@
         <v>2</v>
       </c>
       <c r="AV198">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW198">
         <v>6</v>
@@ -43487,7 +43490,7 @@
         <v>3</v>
       </c>
       <c r="AV207">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW207">
         <v>14</v>
@@ -44687,7 +44690,7 @@
         <v>3</v>
       </c>
       <c r="AV213">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW213">
         <v>2</v>
@@ -44887,7 +44890,7 @@
         <v>3</v>
       </c>
       <c r="AV214">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW214">
         <v>1</v>
@@ -45287,7 +45290,7 @@
         <v>2</v>
       </c>
       <c r="AV216">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW216">
         <v>22</v>
@@ -45487,7 +45490,7 @@
         <v>3</v>
       </c>
       <c r="AV217">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW217">
         <v>4</v>
@@ -46887,7 +46890,7 @@
         <v>3</v>
       </c>
       <c r="AV224">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AW224">
         <v>4</v>
@@ -47887,7 +47890,7 @@
         <v>4</v>
       </c>
       <c r="AV229">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW229">
         <v>14</v>
@@ -48687,7 +48690,7 @@
         <v>4</v>
       </c>
       <c r="AV233">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW233">
         <v>11</v>
@@ -50287,7 +50290,7 @@
         <v>3</v>
       </c>
       <c r="AV241">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW241">
         <v>9</v>
@@ -51284,7 +51287,7 @@
         <v>1</v>
       </c>
       <c r="AV246">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW246">
         <v>12</v>
@@ -51484,7 +51487,7 @@
         <v>3</v>
       </c>
       <c r="AV247">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW247">
         <v>13</v>
@@ -52284,7 +52287,7 @@
         <v>3</v>
       </c>
       <c r="AV251">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW251">
         <v>7</v>
@@ -52884,7 +52887,7 @@
         <v>3</v>
       </c>
       <c r="AV254">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW254">
         <v>13</v>
@@ -54881,7 +54884,7 @@
         <v>2</v>
       </c>
       <c r="AV264">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW264">
         <v>13</v>
@@ -55081,7 +55084,7 @@
         <v>3</v>
       </c>
       <c r="AV265">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW265">
         <v>1</v>
@@ -56281,7 +56284,7 @@
         <v>1</v>
       </c>
       <c r="AV271">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW271">
         <v>12</v>
@@ -57281,7 +57284,7 @@
         <v>3</v>
       </c>
       <c r="AV276">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW276">
         <v>23</v>
@@ -58281,7 +58284,7 @@
         <v>3</v>
       </c>
       <c r="AV281">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW281">
         <v>11</v>
@@ -58881,7 +58884,7 @@
         <v>3</v>
       </c>
       <c r="AV284">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW284">
         <v>15</v>
@@ -59681,7 +59684,7 @@
         <v>3</v>
       </c>
       <c r="AV288">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW288">
         <v>6</v>
@@ -60281,7 +60284,7 @@
         <v>2</v>
       </c>
       <c r="AV291">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW291">
         <v>3</v>
@@ -60481,7 +60484,7 @@
         <v>3</v>
       </c>
       <c r="AV292">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW292">
         <v>8</v>
@@ -60881,7 +60884,7 @@
         <v>2</v>
       </c>
       <c r="AV294">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW294">
         <v>6</v>
@@ -64081,7 +64084,7 @@
         <v>2</v>
       </c>
       <c r="AV310">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW310">
         <v>13</v>
@@ -64681,7 +64684,7 @@
         <v>3</v>
       </c>
       <c r="AV313">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW313">
         <v>16</v>
@@ -65281,7 +65284,7 @@
         <v>3</v>
       </c>
       <c r="AV316">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW316">
         <v>6</v>
@@ -66881,7 +66884,7 @@
         <v>3</v>
       </c>
       <c r="AV324">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW324">
         <v>8</v>
@@ -67081,7 +67084,7 @@
         <v>2</v>
       </c>
       <c r="AV325">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW325">
         <v>1</v>
@@ -67881,7 +67884,7 @@
         <v>1</v>
       </c>
       <c r="AV329">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW329">
         <v>9</v>
@@ -68081,7 +68084,7 @@
         <v>4</v>
       </c>
       <c r="AV330">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW330">
         <v>12</v>
@@ -69081,7 +69084,7 @@
         <v>5</v>
       </c>
       <c r="AV335">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW335">
         <v>8</v>
@@ -69281,7 +69284,7 @@
         <v>2</v>
       </c>
       <c r="AV336">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW336">
         <v>13</v>
@@ -69481,7 +69484,7 @@
         <v>3</v>
       </c>
       <c r="AV337">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW337">
         <v>8</v>
@@ -69681,7 +69684,7 @@
         <v>2</v>
       </c>
       <c r="AV338">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW338">
         <v>15</v>
@@ -70281,7 +70284,7 @@
         <v>3</v>
       </c>
       <c r="AV341">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW341">
         <v>4</v>
@@ -70881,7 +70884,7 @@
         <v>5</v>
       </c>
       <c r="AV344">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW344">
         <v>1</v>
@@ -71081,7 +71084,7 @@
         <v>4</v>
       </c>
       <c r="AV345">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW345">
         <v>8</v>
@@ -71281,7 +71284,7 @@
         <v>4</v>
       </c>
       <c r="AV346">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW346">
         <v>10</v>
@@ -71881,7 +71884,7 @@
         <v>4</v>
       </c>
       <c r="AV349">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW349">
         <v>10</v>
@@ -72681,7 +72684,7 @@
         <v>3</v>
       </c>
       <c r="AV353">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW353">
         <v>3</v>
@@ -72881,7 +72884,7 @@
         <v>3</v>
       </c>
       <c r="AV354">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW354">
         <v>3</v>
@@ -73081,7 +73084,7 @@
         <v>3</v>
       </c>
       <c r="AV355">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW355">
         <v>12</v>
@@ -74681,7 +74684,7 @@
         <v>4</v>
       </c>
       <c r="AV363">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW363">
         <v>16</v>
@@ -75281,7 +75284,7 @@
         <v>3</v>
       </c>
       <c r="AV366">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW366">
         <v>16</v>
@@ -76081,7 +76084,7 @@
         <v>3</v>
       </c>
       <c r="AV370">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW370">
         <v>11</v>
@@ -76480,6 +76483,9 @@
       <c r="AU372">
         <v>5</v>
       </c>
+      <c r="AV372">
+        <v>1</v>
+      </c>
       <c r="AW372">
         <v>17</v>
       </c>
@@ -77078,7 +77084,7 @@
         <v>3</v>
       </c>
       <c r="AV375">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW375">
         <v>11</v>
@@ -77278,7 +77284,7 @@
         <v>2</v>
       </c>
       <c r="AV376">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW376">
         <v>6</v>
@@ -79875,7 +79881,7 @@
         <v>1</v>
       </c>
       <c r="AV389">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW389">
         <v>17</v>
@@ -81875,7 +81881,7 @@
         <v>1</v>
       </c>
       <c r="AV399">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW399">
         <v>6</v>
@@ -82275,7 +82281,7 @@
         <v>4</v>
       </c>
       <c r="AV401">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW401">
         <v>15</v>
@@ -82475,7 +82481,7 @@
         <v>4</v>
       </c>
       <c r="AV402">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW402">
         <v>5</v>
@@ -82675,7 +82681,7 @@
         <v>3</v>
       </c>
       <c r="AV403">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW403">
         <v>8</v>
@@ -83075,7 +83081,7 @@
         <v>3</v>
       </c>
       <c r="AV405">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW405">
         <v>14</v>
@@ -83275,7 +83281,7 @@
         <v>3</v>
       </c>
       <c r="AV406">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW406">
         <v>1</v>
@@ -84074,6 +84080,9 @@
       <c r="AU410">
         <v>3</v>
       </c>
+      <c r="AV410">
+        <v>2</v>
+      </c>
       <c r="AW410">
         <v>10</v>
       </c>
@@ -85472,7 +85481,7 @@
         <v>5</v>
       </c>
       <c r="AV417">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW417">
         <v>5</v>
@@ -86072,7 +86081,7 @@
         <v>3</v>
       </c>
       <c r="AV420">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW420">
         <v>11</v>
@@ -86672,7 +86681,7 @@
         <v>3</v>
       </c>
       <c r="AV423">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW423">
         <v>6</v>
@@ -86872,7 +86881,7 @@
         <v>3</v>
       </c>
       <c r="AV424">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW424">
         <v>1</v>
@@ -87272,7 +87281,7 @@
         <v>4</v>
       </c>
       <c r="AV426">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW426">
         <v>12</v>
@@ -87872,7 +87881,7 @@
         <v>3</v>
       </c>
       <c r="AV429">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW429">
         <v>17</v>
@@ -88672,7 +88681,7 @@
         <v>1</v>
       </c>
       <c r="AV433">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW433">
         <v>9</v>
@@ -89072,7 +89081,7 @@
         <v>4</v>
       </c>
       <c r="AV435">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW435">
         <v>13</v>
@@ -89472,7 +89481,7 @@
         <v>3</v>
       </c>
       <c r="AV437">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW437">
         <v>9</v>

</xml_diff>